<commit_message>
Small update on HHC Work
</commit_message>
<xml_diff>
--- a/Design Work/HHC/Prelim HHC BOM.xlsx
+++ b/Design Work/HHC/Prelim HHC BOM.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\nate\Downloads\Cathode Stuff\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\PerytonElectricPropulsion\Design Work\HHC\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7ACE8997-9C76-4A13-B719-9DB7D1D3E321}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E94D97D9-B702-4A67-AB9C-D6E5EBDF7D59}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{FBC354F0-549C-4B23-AB67-491F45504AF1}"/>
   </bookViews>
@@ -469,18 +469,18 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6B9AF862-C870-4A4E-92EE-F0EC8A6F7476}">
-  <dimension ref="A1:C11"/>
+  <dimension ref="A1:K11"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="57.54296875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -491,12 +491,12 @@
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>2</v>
       </c>
@@ -506,8 +506,9 @@
       <c r="C4" s="1" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="K4" s="1"/>
+    </row>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>16</v>
       </c>
@@ -518,7 +519,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>7</v>
       </c>
@@ -528,8 +529,9 @@
       <c r="C6" s="1" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="K6" s="1"/>
+    </row>
+    <row r="7" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>13</v>
       </c>
@@ -540,22 +542,22 @@
         <v>9</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>12</v>
       </c>

</xml_diff>